<commit_message>
test-evidence: add M1-S2 unit test evidence
</commit_message>
<xml_diff>
--- a/test-evidence/M1-Tong-Mingxuan/UT-M1-table.xlsx
+++ b/test-evidence/M1-Tong-Mingxuan/UT-M1-table.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -198,6 +198,60 @@
   </si>
   <si>
     <t>Captured redirect URL equals expected path for each authority (3 cases).</t>
+  </si>
+  <si>
+    <t>UT-M1-S2-01</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>ProfileController + MockMvc; UserRepository mocked to return existing logged-in user; save returns updated user.</t>
+  </si>
+  <si>
+    <t>POST /profile with principal student1@student.xjtlu.edu.cn, name=Student One Updated, phone=18812345678, department=Computer Science.</t>
+  </si>
+  <si>
+    <t>HTTP 302 redirect to /profile?success=true; userRepository.save called once.</t>
+  </si>
+  <si>
+    <t>When valid data is submitted, profile should be persisted and success feedback should be available on redirect.</t>
+  </si>
+  <si>
+    <t>Redirect URL matches and save(...) invocation verified once in ProfileControllerTest.</t>
+  </si>
+  <si>
+    <t>UT-M1-S2-02</t>
+  </si>
+  <si>
+    <t>ProfileController + MockMvc; UserRepository mocked with existing user.</t>
+  </si>
+  <si>
+    <t>POST /profile with phone empty, department non-empty (other fields valid).</t>
+  </si>
+  <si>
+    <t>HTTP 200 returns profile view; model has field error on profileForm.phone with code NotBlank; save not called.</t>
+  </si>
+  <si>
+    <t>Mandatory Phone Number cannot be empty; saving must be blocked and Field is required warning shown.</t>
+  </si>
+  <si>
+    <t>Field error for phone asserted and verify(save, never()) passed.</t>
+  </si>
+  <si>
+    <t>UT-M1-S2-03</t>
+  </si>
+  <si>
+    <t>POST /profile with department empty, phone non-empty (other fields valid).</t>
+  </si>
+  <si>
+    <t>HTTP 200 returns profile view; model has field error on profileForm.department with code NotBlank; save not called.</t>
+  </si>
+  <si>
+    <t>Mandatory Department cannot be empty; saving must be blocked and Field is required warning shown.</t>
+  </si>
+  <si>
+    <t>Field error for department asserted and verify(save, never()) passed.</t>
   </si>
 </sst>
 </file>
@@ -210,7 +264,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,13 +286,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -383,7 +430,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -447,12 +494,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -713,209 +754,173 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -995,8 +1000,6 @@
     <dxf>
       <font>
         <b val="1"/>
-        <i val="0"/>
-        <u val="none"/>
         <sz val="11"/>
         <color rgb="FF08090C"/>
       </font>
@@ -1017,8 +1020,6 @@
     <dxf>
       <font>
         <b val="1"/>
-        <i val="0"/>
-        <u val="none"/>
         <sz val="11"/>
         <color rgb="FF08090C"/>
       </font>
@@ -1039,8 +1040,6 @@
     <dxf>
       <font>
         <b val="1"/>
-        <i val="0"/>
-        <u val="none"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
       </font>
@@ -1065,8 +1064,6 @@
     <dxf>
       <font>
         <b val="1"/>
-        <i val="0"/>
-        <u val="none"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
       </font>
@@ -1086,9 +1083,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <u val="none"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
       </font>
@@ -1112,7 +1106,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="中色系标题行镶边行表格样式_6e22f3" count="7" xr9:uid="{C45723AE-D397-44DA-BB19-79410AAD38E5}">
+    <tableStyle name="中色系标题行镶边行表格样式_6e22f3" count="7" xr9:uid="{80F17A25-D776-48CA-A2B7-6825C5CD7F31}">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -1415,7 +1409,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.5663716814159" customWidth="1"/>
@@ -1428,235 +1422,323 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="65" customHeight="1" spans="1:8">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1" spans="1:8">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" ht="73" customHeight="1" spans="1:8">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" ht="67" customHeight="1" spans="1:8">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" ht="69" customHeight="1" spans="1:8">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" ht="55.5" customHeight="1" spans="1:8">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" ht="39" customHeight="1" spans="1:8">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1" spans="1:8">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="6" t="s">
         <v>15</v>
       </c>
+    </row>
+    <row r="10" ht="60" spans="1:8">
+      <c r="A10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" ht="45" spans="1:8">
+      <c r="A11" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" ht="45" spans="1:8">
+      <c r="A12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" ht="15" spans="1:8">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test-evidence: add PBI1.5 unit test evidence
</commit_message>
<xml_diff>
--- a/test-evidence/M1-Tong-Mingxuan/UT-M1-table.xlsx
+++ b/test-evidence/M1-Tong-Mingxuan/UT-M1-table.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="111">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -252,6 +252,114 @@
   </si>
   <si>
     <t>Field error for department asserted and verify(save, never()) passed.</t>
+  </si>
+  <si>
+    <t>UT-M1-S3-01</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>PasswordResetService under test; UserRepository and EmailService mocked; tokenRepository.save returns the same token instance.</t>
+  </si>
+  <si>
+    <t>PasswordResetService.createResetTokenAndSendEmail("s@student.xjtlu.edu.cn") where user exists in DB.</t>
+  </si>
+  <si>
+    <t>PasswordResetToken saved with: user=existing user, token=non-blank UUID, expiresAt &gt; now, used=false; EmailService.sendPasswordResetEmail called with same email and token.</t>
+  </si>
+  <si>
+    <t>For a registered email, system creates a reset token with 30-minute expiry and triggers email sending.</t>
+  </si>
+  <si>
+    <t>Token saved with correct user, non-blank token, future expiry, used=false; emailService.sendPasswordResetEmail verified with matching arguments.</t>
+  </si>
+  <si>
+    <t>UT-M1-S3-02</t>
+  </si>
+  <si>
+    <t>PasswordResetService under test; tokenRepository returns a valid token (used=false, expires 10min from now); passwordEncoder.encode("newPass") returns "new-hash".</t>
+  </si>
+  <si>
+    <t>PasswordResetService.validateTokenAndResetPassword("abc", "newPass")</t>
+  </si>
+  <si>
+    <t>Returns null (no error); user.passwordHash = "new-hash"; token.used = true; userRepository and tokenRepository save called.</t>
+  </si>
+  <si>
+    <t>Valid reset token updates the user password and marks token as used to prevent reuse.</t>
+  </si>
+  <si>
+    <t>assertNull(error); assertEquals("new-hash", user.getPasswordHash()); assertTrue(token.getUsed()); verify save on both repositories.</t>
+  </si>
+  <si>
+    <t>UT-M1-S3-03</t>
+  </si>
+  <si>
+    <t>PasswordResetService under test; tokenRepository returns empty for token "invalid".</t>
+  </si>
+  <si>
+    <t>PasswordResetService.validateTokenAndResetPassword("invalid", "newPass")</t>
+  </si>
+  <si>
+    <t>Returns "Invalid reset link."; userRepository.save never called.</t>
+  </si>
+  <si>
+    <t>A non-existent or invalid token results in an error and no password update.</t>
+  </si>
+  <si>
+    <t>assertEquals("Invalid reset link.", error); verify(userRepository, never()).save(any()).</t>
+  </si>
+  <si>
+    <t>UT-M1-S3-04</t>
+  </si>
+  <si>
+    <t>PasswordResetController + MockMvc; filters disabled; PasswordResetService mocked.</t>
+  </si>
+  <si>
+    <t>POST /forgot-password with email=s@student.xjtlu.edu.cn.</t>
+  </si>
+  <si>
+    <t>HTTP 302 redirect to /forgot-password; flash attribute "infoMessage" exists; service.createResetTokenAndSendEmail called with same email.</t>
+  </si>
+  <si>
+    <t>Submitting an email triggers the reset token flow and shows a generic info message (does not reveal whether email exists).</t>
+  </si>
+  <si>
+    <t>Redirect URL, flash attribute, and verify(service).createResetTokenAndSendEmail("s@student.xjtlu.edu.cn") match expectations.</t>
+  </si>
+  <si>
+    <t>UT-M1-S3-05</t>
+  </si>
+  <si>
+    <t>POST /reset-password with token=abc, password=newPass1, confirmPassword=newPass2 (mismatched).</t>
+  </si>
+  <si>
+    <t>HTTP 200; view name = "reset-password"; model attribute "errorMessage" = "Passwords do not match."</t>
+  </si>
+  <si>
+    <t>When new password and confirm password do not match, the system shows "Passwords do not match" error and does not proceed.</t>
+  </si>
+  <si>
+    <t>status().isOk(); model().attribute("errorMessage", "Passwords do not match.") as asserted.</t>
+  </si>
+  <si>
+    <t>UT-M1-S3-06</t>
+  </si>
+  <si>
+    <t>PasswordResetController + MockMvc; filters disabled; PasswordResetService mocked; validateTokenAndResetPassword returns null (success).</t>
+  </si>
+  <si>
+    <t>POST /reset-password with token=valid-token, password=newPassword, confirmPassword=newPassword.</t>
+  </si>
+  <si>
+    <t>HTTP 302 redirect to /login?reset=true; service.validateTokenAndResetPassword called with ("valid-token", "newPassword").</t>
+  </si>
+  <si>
+    <t>Successful password reset redirects to login page with reset=true parameter, showing a success message.</t>
+  </si>
+  <si>
+    <t>redirectedUrl("/login?reset=true"); verify(service).validateTokenAndResetPassword("valid-token", "newPassword") match expectations.</t>
   </si>
 </sst>
 </file>
@@ -1106,7 +1214,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="中色系标题行镶边行表格样式_6e22f3" count="7" xr9:uid="{80F17A25-D776-48CA-A2B7-6825C5CD7F31}">
+    <tableStyle name="中色系标题行镶边行表格样式_6e22f3" count="7" xr9:uid="{81F29B1D-7238-4530-A4E9-1CCB41305B90}">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -1409,7 +1517,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.5663716814159" customWidth="1"/>
@@ -1652,7 +1760,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" ht="60" spans="1:8">
+    <row r="10" ht="60" customHeight="1" spans="1:8">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
@@ -1678,7 +1786,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" ht="45" spans="1:8">
+    <row r="11" ht="45" customHeight="1" spans="1:8">
       <c r="A11" s="6" t="s">
         <v>64</v>
       </c>
@@ -1704,7 +1812,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" ht="45" spans="1:8">
+    <row r="12" ht="45" customHeight="1" spans="1:8">
       <c r="A12" s="2" t="s">
         <v>70</v>
       </c>
@@ -1730,15 +1838,161 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" ht="15" spans="1:8">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+    <row r="13" ht="45" customHeight="1" spans="1:8">
+      <c r="A13" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1" spans="1:8">
+      <c r="A14" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1" spans="1:8">
+      <c r="A15" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1" spans="1:8">
+      <c r="A16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1" spans="1:8">
+      <c r="A17" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1" spans="1:8">
+      <c r="A18" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>